<commit_message>
major changes to code
</commit_message>
<xml_diff>
--- a/wenzhounese_video_log (1).xlsx
+++ b/wenzhounese_video_log (1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eason\Jordan Stuff\项目\Survey\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eason\Jordan Stuff\项目\Survey - 副本\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73ADA96C-CCFA-4634-B3FC-1E631B945D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB69057C-077A-4F7F-AEE7-A51B5424C9FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="852" windowWidth="21600" windowHeight="11232" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Video Log" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="262">
   <si>
     <t>🗂️  DROPDOWN VALUES — WHAT EACH OPTION MEANS</t>
   </si>
@@ -781,6 +781,190 @@
   </si>
   <si>
     <t>target_aa</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>温州娃不会讲温州话，在意大利的温州娃却会讲温州话</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>#温州#百晓二姐#意大利温州人</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.douyin.com/video/7653065391829472683</t>
+  </si>
+  <si>
+    <t>百晓二姐</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>target_ab</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.douyin.com/video/7654436433196763078</t>
+  </si>
+  <si>
+    <r>
+      <t>来听听意大利侨二代温州话说得怎么样</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>#温州#百晓二姐#意大利温州人</t>
+    </r>
+  </si>
+  <si>
+    <t>在欧洲，很多老外不会普通话，但是会学会温州话！因为温州人已经把欧洲温州化。。。哈哈哈哈</t>
+  </si>
+  <si>
+    <t>https://www.douyin.com/video/7440391398479744313</t>
+  </si>
+  <si>
+    <t>全能朱大定居法国</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.douyin.com/video/6873023993050402062</t>
+  </si>
+  <si>
+    <r>
+      <t>第1集 | 用温州话打开</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>#小猪佩奇</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>OT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>老师</t>
+    </r>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>target_ac</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>target_ad</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>target_ae</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.douyin.com/video/7260065560329817344</t>
+  </si>
+  <si>
+    <r>
+      <t>#温州童谣</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>#打珓杯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>#温州话</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>#温州</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>#温州方言</t>
+    </r>
+  </si>
+  <si>
+    <t>炳松频道</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>target_ag</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
 </sst>
@@ -788,7 +972,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -860,6 +1044,29 @@
       <b/>
       <sz val="9"/>
       <color rgb="FF1F3864"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -965,7 +1172,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -996,6 +1203,17 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1273,6 +1491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:T53"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1293,61 +1512,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13"/>
-      <c r="P1" s="13"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
+      <c r="P1" s="18"/>
       <c r="Q1" s="7"/>
     </row>
     <row r="2" spans="1:20" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="12" t="s">
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="12" t="s">
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
-      <c r="K2" s="12" t="s">
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="L2" s="13"/>
-      <c r="M2" s="12" t="s">
+      <c r="L2" s="18"/>
+      <c r="M2" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="N2" s="13"/>
-      <c r="O2" s="12" t="s">
+      <c r="N2" s="18"/>
+      <c r="O2" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="12" t="s">
+      <c r="P2" s="18"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="S2" s="13"/>
-      <c r="T2" s="13"/>
+      <c r="S2" s="18"/>
+      <c r="T2" s="18"/>
     </row>
     <row r="3" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -2690,10 +2909,16 @@
       <c r="A36" s="2">
         <v>33</v>
       </c>
-      <c r="B36" s="2"/>
+      <c r="B36" s="2" t="s">
+        <v>244</v>
+      </c>
       <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
+      <c r="D36" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="E36" s="2">
+        <v>36</v>
+      </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
@@ -2701,20 +2926,37 @@
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
-      <c r="M36" s="2"/>
+      <c r="M36" s="13" t="s">
+        <v>245</v>
+      </c>
       <c r="N36" s="2"/>
-      <c r="O36" s="2"/>
-      <c r="P36" s="2"/>
-      <c r="Q36" s="2"/>
+      <c r="O36" s="2">
+        <v>572</v>
+      </c>
+      <c r="P36" s="2">
+        <v>16</v>
+      </c>
+      <c r="Q36" s="2">
+        <v>40</v>
+      </c>
+      <c r="R36" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="37" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>34</v>
       </c>
-      <c r="B37" s="3"/>
+      <c r="B37" s="3" t="s">
+        <v>247</v>
+      </c>
       <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
+      <c r="D37" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="E37" s="3">
+        <v>29</v>
+      </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
@@ -2722,20 +2964,37 @@
       <c r="J37" s="3"/>
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
-      <c r="M37" s="3"/>
+      <c r="M37" s="13" t="s">
+        <v>245</v>
+      </c>
       <c r="N37" s="3"/>
-      <c r="O37" s="3"/>
-      <c r="P37" s="3"/>
-      <c r="Q37" s="3"/>
+      <c r="O37" s="3">
+        <v>1093</v>
+      </c>
+      <c r="P37" s="3">
+        <v>85</v>
+      </c>
+      <c r="Q37" s="3">
+        <v>270</v>
+      </c>
+      <c r="R37" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="38" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>35</v>
       </c>
-      <c r="B38" s="2"/>
+      <c r="B38" s="2" t="s">
+        <v>250</v>
+      </c>
       <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
+      <c r="D38" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="E38" s="2">
+        <v>57</v>
+      </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
@@ -2743,20 +3002,37 @@
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
-      <c r="M38" s="2"/>
+      <c r="M38" s="13" t="s">
+        <v>251</v>
+      </c>
       <c r="N38" s="2"/>
-      <c r="O38" s="2"/>
-      <c r="P38" s="2"/>
-      <c r="Q38" s="2"/>
+      <c r="O38" s="2">
+        <v>22000</v>
+      </c>
+      <c r="P38" s="2">
+        <v>3142</v>
+      </c>
+      <c r="Q38" s="2">
+        <v>33000</v>
+      </c>
+      <c r="R38" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="39" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>36</v>
       </c>
-      <c r="B39" s="3"/>
+      <c r="B39" s="3" t="s">
+        <v>252</v>
+      </c>
       <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
+      <c r="D39" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="E39" s="3">
+        <v>20</v>
+      </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
@@ -2764,11 +3040,22 @@
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
-      <c r="M39" s="3"/>
+      <c r="M39" s="14" t="s">
+        <v>254</v>
+      </c>
       <c r="N39" s="3"/>
-      <c r="O39" s="3"/>
-      <c r="P39" s="3"/>
-      <c r="Q39" s="3"/>
+      <c r="O39" s="3">
+        <v>4993</v>
+      </c>
+      <c r="P39" s="3">
+        <v>1275</v>
+      </c>
+      <c r="Q39" s="3">
+        <v>5480</v>
+      </c>
+      <c r="R39" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="40" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
@@ -2776,7 +3063,7 @@
       </c>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
+      <c r="D40" s="12"/>
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
@@ -2785,7 +3072,7 @@
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
       <c r="L40" s="2"/>
-      <c r="M40" s="2"/>
+      <c r="M40" s="13"/>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
       <c r="P40" s="2"/>
@@ -2795,10 +3082,16 @@
       <c r="A41" s="3">
         <v>38</v>
       </c>
-      <c r="B41" s="3"/>
+      <c r="B41" s="3" t="s">
+        <v>258</v>
+      </c>
       <c r="C41" s="3"/>
-      <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
+      <c r="D41" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="E41" s="3">
+        <v>74</v>
+      </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
@@ -2806,11 +3099,22 @@
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
-      <c r="M41" s="3"/>
+      <c r="M41" s="16" t="s">
+        <v>260</v>
+      </c>
       <c r="N41" s="3"/>
-      <c r="O41" s="3"/>
-      <c r="P41" s="3"/>
-      <c r="Q41" s="3"/>
+      <c r="O41" s="3">
+        <v>7825</v>
+      </c>
+      <c r="P41" s="3">
+        <v>1337</v>
+      </c>
+      <c r="Q41" s="3">
+        <v>4497</v>
+      </c>
+      <c r="R41" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="42" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
@@ -3121,11 +3425,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
     </row>
     <row r="2" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
@@ -3335,11 +3639,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
     </row>
     <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">

</xml_diff>